<commit_message>
Add comprehensive parameter loading documentation
Co-authored-by: bi-kash <32809050+bi-kash@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/strategy_parameters_template.xlsx
+++ b/strategy_parameters_template.xlsx
@@ -482,14 +482,13 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>Min Gap Percent</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>70</v>
+        <v>150</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -503,7 +502,6 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>Target Retrace Percent</t>
@@ -524,7 +522,6 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>Max Float Millions</t>
@@ -545,7 +542,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>Min Volume Millions</t>
@@ -591,7 +587,6 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
           <t>Min Green Days</t>
@@ -612,7 +607,6 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>Max Float Millions</t>
@@ -633,7 +627,6 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
           <t>Min Volume Millions</t>
@@ -679,7 +672,6 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
           <t>Min Gap Down Percent</t>
@@ -700,7 +692,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
           <t>Max Float Millions</t>
@@ -721,7 +712,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
           <t>Min Volume Millions</t>
@@ -767,7 +757,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
           <t>Min Gap Percent</t>
@@ -788,7 +777,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
           <t>Entry Time</t>
@@ -811,7 +799,6 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
           <t>Min Volume Millions</t>
@@ -857,7 +844,6 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
           <t>Min Volume Ratio</t>
@@ -878,7 +864,6 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
           <t>Min Volume Millions</t>
@@ -899,7 +884,6 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
           <t>Breakout Period Days</t>
@@ -930,7 +914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -943,66 +927,131 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1. Modify the "Current Value" column to change strategy parameters</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2. Save this file</t>
-        </is>
-      </c>
-    </row>
+          <t>🎯 HOW TO USE THIS FILE FOR BACKTESTING:</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3. The backtest system will read these parameters</t>
+          <t>1. Modify the "Current Value" column to change strategy parameters</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>4. Higher gap percentages = more selective but potentially more profitable</t>
+          <t>2. Save this file</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>5. Lower float = more volatile stocks</t>
+          <t>3. RESTART the program (python main.py)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>6. Higher volume = more liquid stocks</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>7. Test different combinations to optimize performance</t>
-        </is>
-      </c>
-    </row>
+          <t>4. Run backtest - the system will automatically use these parameters!</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>📌 IMPORTANT NOTES:</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>IMPORTANT: Only modify the "Current Value" column!</t>
+          <t>• Parameters are loaded when the program STARTS</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>• Changes take effect AFTER restarting the program</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>• If this file exists, Excel parameters are used (NOT config.py)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>• To use config.py instead, delete or rename this Excel file</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>💡 PARAMETER TIPS:</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>• Higher gap percentages = more selective (fewer signals)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>• Lower float = more volatile stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>• Higher volume = more liquid stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>• Test different combinations to optimize performance</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>⚠️ IMPORTANT: Only modify the "Current Value" column!</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>Keep all other columns unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>📖 See PARAMETER_LOADING.md for complete documentation.</t>
         </is>
       </c>
     </row>

</xml_diff>